<commit_message>
Update pricing document and test leads sheet
</commit_message>
<xml_diff>
--- a/test_leads.xlsx
+++ b/test_leads.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\siddhu_surineni\Downloads\eduction\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\siddhu_surineni\Downloads\eduction\eduction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC2BF7E2-ED60-42B3-AECA-9E92875867B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C5272FA-E584-49E2-BB2A-DCCF63F66117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2620" yWindow="2620" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>Name</t>
   </si>
@@ -53,9 +53,6 @@
     <t>+916300130119</t>
   </si>
   <si>
-    <t>siddhu.s@example.com</t>
-  </si>
-  <si>
     <t>john.doe@example.com</t>
   </si>
   <si>
@@ -68,17 +65,31 @@
     <t>Interested</t>
   </si>
   <si>
-    <t>nagendra</t>
+    <t>2003A5201@gamail.com</t>
+  </si>
+  <si>
+    <t>amulya</t>
+  </si>
+  <si>
+    <t>Vennela</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -101,13 +112,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -408,11 +422,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="13.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -436,39 +451,53 @@
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
-        <v>6</v>
+      <c r="C2" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>919885803847</v>
       </c>
       <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
         <v>7</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>7981725896</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B4">
-        <v>917702030136</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
+      <c r="B5">
+        <v>9441674674</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{3694592B-3F1E-41F7-8FF8-BF8D06B157DA}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>